<commit_message>
Nuevos controles y Consulta 17-08
</commit_message>
<xml_diff>
--- a/bases/CNO.xlsx
+++ b/bases/CNO.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="145">
   <si>
     <t>OCU</t>
   </si>
@@ -41,324 +41,159 @@
     <t>Tarea</t>
   </si>
   <si>
-    <t>00. Funcionarios del poder ejecutivo nacional, provincial, municipal y/o departamental</t>
-  </si>
-  <si>
     <t>01</t>
   </si>
   <si>
-    <t>01. Funcionarios del poder legislativo nacional, provincial, municipal y/o departamental</t>
-  </si>
-  <si>
     <t>02</t>
   </si>
   <si>
-    <t>02. Funcionarios del poder judicial federal, nacional, provincial, municipal y/ o departamental</t>
-  </si>
-  <si>
     <t>03</t>
   </si>
   <si>
-    <t>03. Directivos de organismos, empresas e instituciones estatales</t>
-  </si>
-  <si>
     <t>04</t>
   </si>
   <si>
-    <t>04. Directivos de instituciones sociales (comunales, políticas, gremiales, religiosas, derechos humanos, medio ambiente y otras instituciones de bien público)</t>
-  </si>
-  <si>
     <t>05</t>
   </si>
   <si>
-    <t>05. Directivos de pequeñas empresas y microempresas (patrones de 1 a 5 personas)</t>
-  </si>
-  <si>
     <t>06</t>
   </si>
   <si>
-    <t>06. Directivos de medianas empresas privadas productoras de bienes y/o servicios (establecimientos de 6 a 40 personas)</t>
-  </si>
-  <si>
     <t>07</t>
   </si>
   <si>
-    <t>07. Directivos de grandes empresas privadas productoras de bienes y/ o servicios (establecimientos de 41 personas y más)</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
-    <t>10. Ocupaciones de la gestión administrativa, planificación y control de gestión.</t>
-  </si>
-  <si>
     <t>11</t>
   </si>
   <si>
-    <t>11. Ocupaciones de gestión jurídico-legal.</t>
-  </si>
-  <si>
     <t>20</t>
   </si>
   <si>
-    <t>20. Ocupaciones de gestión presupuestaria, contable y financiera:</t>
-  </si>
-  <si>
     <t>30</t>
   </si>
   <si>
-    <t>30. Ocupaciones de la comercialización directa</t>
-  </si>
-  <si>
     <t>31</t>
   </si>
   <si>
-    <t>31. Ocupaciones del corretaje comercial, venta domiciliaria, viajantes y promotores.</t>
-  </si>
-  <si>
     <t>32</t>
   </si>
   <si>
-    <t>32. Ocupaciones de la comercialización indirecta.</t>
-  </si>
-  <si>
-    <t>20. Ocupaciones de gestión presupuestaria, contable y financiera</t>
-  </si>
-  <si>
-    <t>31. Ocupaciones del corretaje comercial, venta domiciliaria, viajantes y promotores</t>
-  </si>
-  <si>
-    <t>32. Ocupaciones de la comercialización indirecta</t>
-  </si>
-  <si>
     <t>33</t>
   </si>
   <si>
-    <t>33. Ocupaciones de la comercialización ambulante y callejera</t>
-  </si>
-  <si>
     <t>34</t>
   </si>
   <si>
-    <t>34. Ocupaciones del transporte</t>
-  </si>
-  <si>
     <t>35</t>
   </si>
   <si>
-    <t>35. Ocupaciones de las telecomunicaciones</t>
-  </si>
-  <si>
     <t>36</t>
   </si>
   <si>
-    <t>36. Ocupaciones del almacenaje</t>
-  </si>
-  <si>
     <t>40</t>
   </si>
   <si>
-    <t>40. Ocupaciones de la salud y sanidad</t>
-  </si>
-  <si>
     <t>41</t>
   </si>
   <si>
-    <t>41. Ocupaciones de la educación</t>
-  </si>
-  <si>
     <t>42</t>
   </si>
   <si>
-    <t>42. Ocupaciones de la investigación científica y tecnológica</t>
-  </si>
-  <si>
     <t>43</t>
   </si>
   <si>
-    <t xml:space="preserve">43. Ocupaciones de la asesoría y consultoría. </t>
-  </si>
-  <si>
     <t>44</t>
   </si>
   <si>
-    <t xml:space="preserve">44. Ocupaciones de prevención de siniestros y atención del medio ambiente y ecología. </t>
-  </si>
-  <si>
     <t>45</t>
   </si>
   <si>
-    <t>45. Ocupaciones de la comunicación de masas.</t>
-  </si>
-  <si>
     <t>46</t>
   </si>
   <si>
-    <t xml:space="preserve">46. Ocupaciones de los servicios sociales, comunales, políticos, gremiales y religiosos. </t>
-  </si>
-  <si>
     <t>47</t>
   </si>
   <si>
-    <t xml:space="preserve">47. Ocupaciones de los servicios de vigilancia y seguridad civil. </t>
-  </si>
-  <si>
     <t>48</t>
   </si>
   <si>
-    <t xml:space="preserve">48. Ocupaciones de servicios policiales. </t>
-  </si>
-  <si>
     <t>49</t>
   </si>
   <si>
-    <t>49. Ocupaciones de las FF.AA., Gendarmería y Prefectura</t>
-  </si>
-  <si>
     <t>50</t>
   </si>
   <si>
-    <t xml:space="preserve">50. Ocupaciones del arte. </t>
-  </si>
-  <si>
     <t>51</t>
   </si>
   <si>
-    <t xml:space="preserve">51. Ocupaciones del deporte. </t>
-  </si>
-  <si>
     <t>52</t>
   </si>
   <si>
-    <t xml:space="preserve">52. Ocupaciones de servicios de recreación. </t>
-  </si>
-  <si>
     <t>53</t>
   </si>
   <si>
-    <t xml:space="preserve">53. Ocupaciones de servicios gastronómicos. </t>
-  </si>
-  <si>
     <t>54</t>
   </si>
   <si>
-    <t xml:space="preserve">54. Ocupaciones del alojamiento y turismo. </t>
-  </si>
-  <si>
     <t>55</t>
   </si>
   <si>
-    <t xml:space="preserve">55. Ocupaciones de servicios domésticos. </t>
-  </si>
-  <si>
     <t>56</t>
   </si>
   <si>
-    <t xml:space="preserve">56. Ocupaciones de servicios de limpieza (no domésticos). </t>
-  </si>
-  <si>
     <t>57</t>
   </si>
   <si>
-    <t xml:space="preserve">57. Ocupaciones del cuidado y la atención de personas. </t>
-  </si>
-  <si>
     <t>58</t>
   </si>
   <si>
-    <t>58. Otras ocupaciones de servicios varios.</t>
-  </si>
-  <si>
     <t>60</t>
   </si>
   <si>
-    <t xml:space="preserve">60. Ocupaciones de la producción agrícola. </t>
-  </si>
-  <si>
     <t>61</t>
   </si>
   <si>
-    <t xml:space="preserve">61. Ocupaciones de la producción ganadera. </t>
-  </si>
-  <si>
     <t>62</t>
   </si>
   <si>
-    <t xml:space="preserve">62. Ocupaciones de la producción forestal. </t>
-  </si>
-  <si>
     <t>63</t>
   </si>
   <si>
-    <t xml:space="preserve">63. Ocupaciones de la producción apícola, avícola y de otras especies menores. </t>
-  </si>
-  <si>
     <t>64</t>
   </si>
   <si>
-    <t xml:space="preserve">64. Ocupaciones de la producción pesquera. </t>
-  </si>
-  <si>
     <t>65</t>
   </si>
   <si>
-    <t>65. Ocupaciones de la caza.</t>
-  </si>
-  <si>
     <t>70</t>
   </si>
   <si>
-    <t xml:space="preserve">70. Ocupaciones de la producción extractiva. </t>
-  </si>
-  <si>
     <t>71</t>
   </si>
   <si>
-    <t xml:space="preserve">71. Ocupaciones de la producción de energía, agua y gas. </t>
-  </si>
-  <si>
     <t>72</t>
   </si>
   <si>
-    <t>72. Ocupaciones de la construcción edilicia y de obras de infraestructura y de redes de distribución de energía, agua potable, gas, telefonía y petróleo</t>
-  </si>
-  <si>
     <t>80</t>
   </si>
   <si>
-    <t xml:space="preserve">80 .Ocupaciones de la producción artesanal e industrial. </t>
-  </si>
-  <si>
     <t>81</t>
   </si>
   <si>
-    <t xml:space="preserve">81. Ocupaciones de la producción de software. </t>
-  </si>
-  <si>
     <t>82</t>
   </si>
   <si>
-    <t>82. Ocupaciones de la reparación de bienes de consumo.</t>
-  </si>
-  <si>
     <t>90</t>
   </si>
   <si>
-    <t xml:space="preserve">90. Ocupaciones de la instalación y mantenimiento de maquinarias, equipos y sistemas de la producción de bienes. </t>
-  </si>
-  <si>
     <t>91</t>
   </si>
   <si>
-    <t xml:space="preserve">91. Ocupaciones del desarrollo tecnológico productivo. </t>
-  </si>
-  <si>
     <t>92</t>
   </si>
   <si>
-    <t>92. Ocupaciones de la instalación y mantenimiento de maquinarias y equipos de la prestación de servicios.</t>
-  </si>
-  <si>
     <t>Jerarquia</t>
   </si>
   <si>
@@ -368,81 +203,111 @@
     <t>Grupo</t>
   </si>
   <si>
-    <t>Ocupaciones de dirección</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
-    <t xml:space="preserve">Ocupaciones de gestión administrativa, de planificación, control de gestión y jurídico-legal </t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
-    <t>Ocupaciones de gestión presupuestaria, contable y financiera</t>
-  </si>
-  <si>
     <t>3</t>
   </si>
   <si>
-    <t>Ocupaciones de comercialización,transporte, telecomunicaciones y almacenaje</t>
-  </si>
-  <si>
     <t>4</t>
   </si>
   <si>
-    <t>Ocupaciones de servicios sociales básicos</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
-    <t>Ocupaciones de servicios varios</t>
-  </si>
-  <si>
     <t>6</t>
   </si>
   <si>
-    <t>Ocupaciones agropecuarias, forestales, de la pesca y de la caza</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
-    <t>Ocupaciones de la producción extractiva, energética, de construcción e infraestructura</t>
-  </si>
-  <si>
     <t>8</t>
   </si>
   <si>
-    <t>Ocupaciones de la producción artesanal, industrial y de reparación de bienes de consumo</t>
-  </si>
-  <si>
     <t>9</t>
   </si>
   <si>
-    <t>Ocupaciones auxiliares de la producción de bienes y la prestación de servicios</t>
-  </si>
-  <si>
     <t>Tecnologia</t>
   </si>
   <si>
-    <t>Ocupaciones sin operación de maquinaria, equipos y sistemas</t>
-  </si>
-  <si>
-    <t>Ocupaciones con operación de maquinaria, equipos o sistemas electromecánicos</t>
-  </si>
-  <si>
-    <t>Ocupaciones con operación de equipos o sistemas informatizados</t>
-  </si>
-  <si>
-    <t>Ocupaciones del desarrollo tecnológico, la instalación y la reparación de maquinaria o equipos</t>
-  </si>
-  <si>
     <t>Calificacion</t>
   </si>
   <si>
+    <t>99</t>
+  </si>
+  <si>
+    <t>No especificada</t>
+  </si>
+  <si>
+    <t>Funcionarios del poder ejecutivo nacional, provincial, municipal y/o departamental</t>
+  </si>
+  <si>
+    <t>Funcionarios del poder legislativo nacional, provincial, municipal y/o departamental</t>
+  </si>
+  <si>
+    <t>Funcionarios del poder judicial federal, nacional, provincial, municipal y/ o departamental</t>
+  </si>
+  <si>
+    <t>Directivos de organismos, empresas e instituciones estatales</t>
+  </si>
+  <si>
+    <t>Directivos de instituciones sociales (comunales, políticas, gremiales, religiosas, derechos humanos, medio ambiente y otras instituciones de bien público)</t>
+  </si>
+  <si>
+    <t>Directivos de pequeñas empresas y microempresas (patrones de 1 a 5 personas)</t>
+  </si>
+  <si>
+    <t>Directivos de medianas empresas privadas productoras de bienes y/o servicios (establecimientos de 6 a 40 personas)</t>
+  </si>
+  <si>
+    <t>Directivos de grandes empresas privadas productoras de bienes y/ o servicios (establecimientos de 41 personas y más)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión administrativa, de planificación, control de gestión y jurídico-legal </t>
+  </si>
+  <si>
+    <t>Gestión presupuestaria, contable y financiera</t>
+  </si>
+  <si>
+    <t>Dirección</t>
+  </si>
+  <si>
+    <t>Comercialización,transporte, telecomunicaciones y almacenaje</t>
+  </si>
+  <si>
+    <t>Servicios sociales básicos</t>
+  </si>
+  <si>
+    <t>Servicios varios</t>
+  </si>
+  <si>
+    <t>Agropecuarias, forestales, de la pesca y de la caza</t>
+  </si>
+  <si>
+    <t>Producción extractiva, energética, de construcción e infraestructura</t>
+  </si>
+  <si>
+    <t>Producción artesanal, industrial y de reparación de bienes de consumo</t>
+  </si>
+  <si>
+    <t>Auxiliares de la producción de bienes y la prestación de servicios</t>
+  </si>
+  <si>
+    <t>Sin operación de maquinaria, equipos y sistemas</t>
+  </si>
+  <si>
+    <t>Operación de maquinaria, equipos o sistemas electromecánicos</t>
+  </si>
+  <si>
+    <t>Operación de equipos o sistemas informatizados</t>
+  </si>
+  <si>
+    <t>Desarrollo tecnológico, la instalación y la reparación de maquinaria o equipos</t>
+  </si>
+  <si>
     <t>Profesional</t>
   </si>
   <si>
@@ -455,22 +320,145 @@
     <t>No calificada</t>
   </si>
   <si>
-    <t>Ocupaciones de jefatura</t>
-  </si>
-  <si>
-    <t>Ocupaciones de ejecución directa</t>
-  </si>
-  <si>
-    <t>Ocupaciones de cuenta propia</t>
-  </si>
-  <si>
-    <t>99</t>
-  </si>
-  <si>
-    <t>99. No especificada</t>
-  </si>
-  <si>
-    <t>No especificada</t>
+    <t>Jefatura</t>
+  </si>
+  <si>
+    <t>Ejecución directa</t>
+  </si>
+  <si>
+    <t>Cuenta propia</t>
+  </si>
+  <si>
+    <t>De la comercialización directa</t>
+  </si>
+  <si>
+    <t>De gestión presupuestaria, contable y financiera</t>
+  </si>
+  <si>
+    <t>Del corretaje comercial, venta domiciliaria, viajantes y promotores</t>
+  </si>
+  <si>
+    <t>De la comercialización indirecta</t>
+  </si>
+  <si>
+    <t>De la comercialización ambulante y callejera</t>
+  </si>
+  <si>
+    <t>Del transporte</t>
+  </si>
+  <si>
+    <t>De las telecomunicaciones</t>
+  </si>
+  <si>
+    <t>Del almacenaje</t>
+  </si>
+  <si>
+    <t>De la salud y sanidad</t>
+  </si>
+  <si>
+    <t>De la educación</t>
+  </si>
+  <si>
+    <t>De la investigación científica y tecnológica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De los servicios de vigilancia y seguridad civil. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">De servicios policiales. </t>
+  </si>
+  <si>
+    <t>De las FF.AA., Gendarmería y Prefectura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Del arte </t>
+  </si>
+  <si>
+    <t>Del deporte</t>
+  </si>
+  <si>
+    <t>De servicios de recreación</t>
+  </si>
+  <si>
+    <t>De servicios gastronómicos</t>
+  </si>
+  <si>
+    <t>Del alojamiento y turismo</t>
+  </si>
+  <si>
+    <t>De servicios domésticos</t>
+  </si>
+  <si>
+    <t>De servicios de limpieza (no domésticos)</t>
+  </si>
+  <si>
+    <t>Del cuidado y la atención de personas</t>
+  </si>
+  <si>
+    <t>Otras ocupaciones de servicios varios</t>
+  </si>
+  <si>
+    <t>De la producción agrícola</t>
+  </si>
+  <si>
+    <t>De la producción ganadera</t>
+  </si>
+  <si>
+    <t>De la producción forestal</t>
+  </si>
+  <si>
+    <t>De la producción apícola, avícola y de otras especies menores</t>
+  </si>
+  <si>
+    <t>De la producción pesquera</t>
+  </si>
+  <si>
+    <t>De la caza</t>
+  </si>
+  <si>
+    <t>De la producción extractiva</t>
+  </si>
+  <si>
+    <t>De la producción de energía, agua y gas</t>
+  </si>
+  <si>
+    <t>De la construcción edilicia y de obras de infraestructura y de redes de distribución de energía, agua potable, gas, telefonía y petróleo</t>
+  </si>
+  <si>
+    <t>De la producción artesanal e industrial</t>
+  </si>
+  <si>
+    <t>De la producción de software</t>
+  </si>
+  <si>
+    <t>De la reparación de bienes de consumo</t>
+  </si>
+  <si>
+    <t>De la instalación y mantenimiento de maquinarias, equipos y sistemas de la producción de bienes</t>
+  </si>
+  <si>
+    <t>Del desarrollo tecnológico productivo</t>
+  </si>
+  <si>
+    <t>De la instalación y mantenimiento de maquinarias y equipos de la prestación de servicios</t>
+  </si>
+  <si>
+    <t>De los servicios sociales, comunales, políticos, gremiales y religiosos</t>
+  </si>
+  <si>
+    <t>De la comunicación de masas</t>
+  </si>
+  <si>
+    <t>De prevención de siniestros y atención del medio ambiente y ecología</t>
+  </si>
+  <si>
+    <t>De la asesoría y consultoría</t>
+  </si>
+  <si>
+    <t>De gestión jurídico-legal</t>
+  </si>
+  <si>
+    <t>De la gestión administrativa, planificación y control de gestión</t>
   </si>
 </sst>
 </file>
@@ -818,7 +806,7 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="5.5703125" customWidth="1"/>
-    <col min="3" max="3" width="141.85546875" customWidth="1"/>
+    <col min="3" max="3" width="140" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -839,8 +827,8 @@
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
+      <c r="C2" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -848,10 +836,10 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -859,10 +847,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -870,10 +858,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
+        <v>7</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -881,10 +869,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>13</v>
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -892,10 +880,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
-        <v>15</v>
+        <v>9</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -903,10 +891,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -914,10 +902,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" t="s">
-        <v>19</v>
+        <v>11</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -925,10 +913,10 @@
         <v>4</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
+        <v>12</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -936,10 +924,10 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" t="s">
-        <v>23</v>
+        <v>13</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -947,10 +935,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" t="s">
-        <v>25</v>
+        <v>14</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -958,10 +946,10 @@
         <v>4</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>27</v>
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -969,10 +957,10 @@
         <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" t="s">
-        <v>29</v>
+        <v>16</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -980,10 +968,10 @@
         <v>4</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" t="s">
-        <v>31</v>
+        <v>17</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -991,10 +979,10 @@
         <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" t="s">
-        <v>32</v>
+        <v>14</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1002,10 +990,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" t="s">
-        <v>27</v>
+        <v>15</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1013,10 +1001,10 @@
         <v>4</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" t="s">
-        <v>33</v>
+        <v>16</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1024,10 +1012,10 @@
         <v>4</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" t="s">
-        <v>34</v>
+        <v>17</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1035,10 +1023,10 @@
         <v>4</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" t="s">
-        <v>36</v>
+        <v>18</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1046,10 +1034,10 @@
         <v>4</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" t="s">
-        <v>38</v>
+        <v>19</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1057,10 +1045,10 @@
         <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" t="s">
-        <v>40</v>
+        <v>20</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1068,10 +1056,10 @@
         <v>4</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" t="s">
-        <v>42</v>
+        <v>21</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -1079,10 +1067,10 @@
         <v>4</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" t="s">
-        <v>44</v>
+        <v>22</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -1090,10 +1078,10 @@
         <v>4</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" t="s">
-        <v>46</v>
+        <v>23</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1101,10 +1089,10 @@
         <v>4</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C26" t="s">
-        <v>48</v>
+        <v>24</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1112,10 +1100,10 @@
         <v>4</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C27" t="s">
-        <v>50</v>
+        <v>25</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1123,10 +1111,10 @@
         <v>4</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C28" t="s">
-        <v>52</v>
+        <v>26</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -1134,10 +1122,10 @@
         <v>4</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C29" t="s">
-        <v>54</v>
+        <v>27</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1145,10 +1133,10 @@
         <v>4</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" t="s">
-        <v>56</v>
+        <v>28</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -1156,10 +1144,10 @@
         <v>4</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C31" t="s">
-        <v>58</v>
+        <v>29</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1167,10 +1155,10 @@
         <v>4</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C32" t="s">
-        <v>60</v>
+        <v>30</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -1178,10 +1166,10 @@
         <v>4</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" t="s">
-        <v>62</v>
+        <v>31</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1189,10 +1177,10 @@
         <v>4</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" t="s">
-        <v>64</v>
+        <v>32</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1200,10 +1188,10 @@
         <v>4</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" t="s">
-        <v>66</v>
+        <v>33</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1211,10 +1199,10 @@
         <v>4</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C36" t="s">
-        <v>68</v>
+        <v>34</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1222,10 +1210,10 @@
         <v>4</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C37" t="s">
-        <v>70</v>
+        <v>35</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1233,10 +1221,10 @@
         <v>4</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C38" t="s">
-        <v>72</v>
+        <v>36</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1244,10 +1232,10 @@
         <v>4</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C39" t="s">
-        <v>74</v>
+        <v>37</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1255,10 +1243,10 @@
         <v>4</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C40" t="s">
-        <v>76</v>
+        <v>38</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1266,10 +1254,10 @@
         <v>4</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C41" t="s">
-        <v>78</v>
+        <v>39</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1277,10 +1265,10 @@
         <v>4</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C42" t="s">
-        <v>80</v>
+        <v>40</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1288,10 +1276,10 @@
         <v>4</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C43" t="s">
-        <v>82</v>
+        <v>41</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1299,10 +1287,10 @@
         <v>4</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C44" t="s">
-        <v>84</v>
+        <v>42</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1310,10 +1298,10 @@
         <v>4</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C45" t="s">
-        <v>86</v>
+        <v>43</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1321,10 +1309,10 @@
         <v>4</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C46" t="s">
-        <v>88</v>
+        <v>44</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1332,10 +1320,10 @@
         <v>4</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C47" t="s">
-        <v>90</v>
+        <v>45</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1343,10 +1331,10 @@
         <v>4</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C48" t="s">
-        <v>92</v>
+        <v>46</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1354,10 +1342,10 @@
         <v>4</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C49" t="s">
-        <v>94</v>
+        <v>47</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1365,10 +1353,10 @@
         <v>4</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C50" t="s">
-        <v>96</v>
+        <v>48</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1376,10 +1364,10 @@
         <v>4</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C51" t="s">
-        <v>98</v>
+        <v>49</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1387,10 +1375,10 @@
         <v>4</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C52" t="s">
-        <v>100</v>
+        <v>50</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1398,10 +1386,10 @@
         <v>4</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C53" t="s">
-        <v>102</v>
+        <v>51</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1409,10 +1397,10 @@
         <v>4</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="C54" t="s">
-        <v>104</v>
+        <v>52</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -1420,10 +1408,10 @@
         <v>4</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C55" t="s">
-        <v>106</v>
+        <v>53</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -1431,10 +1419,10 @@
         <v>4</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C56" t="s">
-        <v>108</v>
+        <v>54</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1442,10 +1430,10 @@
         <v>4</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C57" t="s">
-        <v>110</v>
+        <v>55</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1453,263 +1441,263 @@
         <v>4</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="C58" t="s">
-        <v>147</v>
+        <v>70</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C59" t="s">
-        <v>114</v>
+        <v>57</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C60" t="s">
-        <v>143</v>
+        <v>60</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C61" t="s">
-        <v>144</v>
+        <v>61</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C62" t="s">
-        <v>145</v>
+        <v>59</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C63" t="s">
-        <v>148</v>
+        <v>67</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="C64" t="s">
-        <v>114</v>
+        <v>57</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C65" t="s">
-        <v>116</v>
+        <v>59</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C66" t="s">
-        <v>118</v>
+        <v>60</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C67" t="s">
-        <v>120</v>
+        <v>61</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C68" t="s">
-        <v>122</v>
+        <v>62</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C69" t="s">
-        <v>124</v>
+        <v>63</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C70" t="s">
-        <v>126</v>
+        <v>64</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="C71" t="s">
-        <v>128</v>
+        <v>65</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="C72" t="s">
-        <v>130</v>
+        <v>66</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C73" t="s">
-        <v>132</v>
+        <v>67</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C74" t="s">
-        <v>134</v>
+        <v>59</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C75" t="s">
-        <v>135</v>
+        <v>60</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C76" t="s">
-        <v>136</v>
+        <v>61</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C77" t="s">
-        <v>137</v>
+        <v>62</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C78" t="s">
-        <v>139</v>
+        <v>59</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C79" t="s">
-        <v>140</v>
+        <v>60</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C80" t="s">
-        <v>141</v>
+        <v>61</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C81" t="s">
-        <v>142</v>
+        <v>62</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agrega pestana de ingresos por ocupacion y sexo en Consultar, corrige duplicados en CNO.xlsx y agrega formato pesos a Formatos.R
</commit_message>
<xml_diff>
--- a/bases/CNO.xlsx
+++ b/bases/CNO.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lia\Documents\Trabajo-Final\bases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lpesaresi\Documents\Trabajo-Final\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F18F1B8F-FEAC-44E2-B09F-93D44FD48652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8220"/>
+    <workbookView xWindow="1428" yWindow="1092" windowWidth="20016" windowHeight="10872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CNO" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="145">
   <si>
     <t>OCU</t>
   </si>
@@ -464,7 +465,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -800,16 +801,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C81"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C77"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="5.5703125" customWidth="1"/>
+    <col min="2" max="2" width="5.5546875" customWidth="1"/>
     <col min="3" max="3" width="140" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -820,7 +821,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -831,7 +832,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -842,7 +843,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -853,7 +854,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -864,7 +865,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -875,7 +876,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -886,7 +887,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -897,7 +898,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -908,7 +909,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -919,7 +920,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -930,7 +931,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -941,7 +942,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -952,7 +953,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -963,7 +964,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -974,729 +975,685 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>4</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>4</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>4</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>4</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>4</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>4</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>4</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>4</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>4</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>4</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>4</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>4</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>4</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>4</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>4</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>4</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>4</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>4</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>4</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>4</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>4</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>4</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>4</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>4</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>4</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>4</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>4</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>4</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>4</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>4</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>4</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>4</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>4</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>4</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>4</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>4</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>4</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>4</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>56</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>58</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="C60" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>56</v>
-      </c>
-      <c r="B60" s="2" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>58</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>58</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>56</v>
-      </c>
-      <c r="B61" s="2" t="s">
+      <c r="C62" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>58</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>56</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>56</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="C63" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>58</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>58</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>58</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>58</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>58</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>58</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>59</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>60</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>69</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>69</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
-        <v>69</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>69</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C81" s="2" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>